<commit_message>
Correct five build-status rows against git
Five items I had labelled 'after build 52' shipped IN build 52 - their
commits sit below the release row. Checked with git, not memory.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build-analysis-july24.xlsx
+++ b/docs/FCC-core-55-70/build-analysis-july24.xlsx
@@ -2482,7 +2482,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>BUILT — after build 52</t>
+          <t>BUILT — in build 52 (corrected 2026-08-12 against git)</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>BUILT — after build 52</t>
+          <t>BUILT — in build 52 (corrected 2026-08-12 against git)</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>BUILT — after build 52</t>
+          <t>BUILT — in build 52 (corrected 2026-08-12 against git)</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>BUILT — after build 52</t>
+          <t>BUILT — in build 52 (corrected 2026-08-12 against git)</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>BUILT — after build 52</t>
+          <t>BUILT — in build 52 (corrected 2026-08-12 against git)</t>
         </is>
       </c>
     </row>

</xml_diff>